<commit_message>
Add description of seed_strategy to example files
</commit_message>
<xml_diff>
--- a/src/semeio/fmudesign/examples/fmudesign_ex_montecarlo.xlsx
+++ b/src/semeio/fmudesign/examples/fmudesign_ex_montecarlo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LGAZ/semeio/src/semeio/fmudesign/examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LEVJE/dev_komodo/semeio/src/semeio/fmudesign/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{673E8D27-B7C0-8747-B672-10EBE2B7D661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AF5827-27A7-2F47-91FE-98C0E2F04E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="27180" windowHeight="18420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="general_input" sheetId="1" r:id="rId1"/>
@@ -57,8 +57,18 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>Number of repeated rms_seeds per sensitivity/sensitivity case. 
-This is overridden if the number of realisations is specified in the “numreal” column in designinput.</t>
+          <t xml:space="preserve">Number of repeated rms_seeds per sensitivity/sensitivity case. 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t>This is overridden if the number of realisations is specified in the “numreal” column in designinput.</t>
         </r>
       </text>
     </comment>
@@ -72,10 +82,40 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>Alternatives:
-- default gives seed numbers 1000, 1001, 1002, ...
-- None (seed number is not added as parameter in output spreadsheet) 
-- filename for file with list of seeds in ert/input/distributions/</t>
+          <t xml:space="preserve">Alternatives:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">- default gives seed numbers 1000, 1001, 1002, ...
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">- None (seed number is not added as parameter in output spreadsheet) 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t>- filename for file with list of seeds in ert/input/distributions/</t>
         </r>
       </text>
     </comment>
@@ -89,10 +129,40 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>Alternatives:
-- None
-- name of sheet in this workbook with background parameters
-- Name of external file with background parameters. Must end with .xlsx or .csv and be readable as pandas dataframe with parameter names as column headers. The path can be absolute, or relative (to the location of this file)</t>
+          <t xml:space="preserve">Alternatives:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">- None
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">- name of sheet in this workbook with background parameters
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t>- Name of external file with background parameters. Must end with .xlsx or .csv and be readable as pandas dataframe with parameter names as column headers. The path can be absolute, or relative (to the location of this file)</t>
         </r>
       </text>
     </comment>
@@ -106,9 +176,29 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>Seed user for random number generator (RNG). Alternatives:
- - A number (e.g. a six digit number like 294284) to see the RNG.
- - None. The RNG will not be seeded and analysis will not be reproducible.</t>
+          <t xml:space="preserve">Seed user for random number generator (RNG). Alternatives:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve"> - A number (e.g. a six digit number like 294284) to see the RNG.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve"> - None. The RNG will not be seeded and analysis will not be reproducible.</t>
         </r>
       </text>
     </comment>
@@ -122,9 +212,62 @@
             <family val="2"/>
             <charset val="1"/>
           </rPr>
-          <t>To correlate variables, an algorithm called Iman-Conover is used.
-- If ‘correlation_iterations’ is set to 0, then only Iman-Conover is used.
-- If ‘correlation_iterations’ is a positive integer, then random swaps will be performed to improve the correlation. This takes a bit longer, but typically leads to observec orrelation that is closer to desired correlation, especially when variables are far from Gaussian (normal distribution). A value of 999 is a good starting point.</t>
+          <t xml:space="preserve">To correlate variables, an algorithm called Iman-Conover is used.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">- If ‘correlation_iterations’ is set to 0, then only Iman-Conover is used.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t>- If ‘correlation_iterations’ is a positive integer, then random swaps will be performed to improve the correlation. This takes a bit longer, but typically leads to observec orrelation that is closer to desired correlation, especially when variables are far from Gaussian (normal distribution). A value of 999 is a good starting point.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{FE51B3DD-ECE6-0D4B-B6BD-790F0F43C73A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Controls how parameter setup changes affect Monte Carlo samples:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> -  joint  (default): Adding, removing, or reordering parameters may change samples for other parameters.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">  -  independent : Samples for unchanged parameters and correlation groups stay the same, provided neither distribution_seed nor the sample size changes. </t>
         </r>
       </text>
     </comment>
@@ -820,7 +963,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="68">
   <si>
     <t>designtype</t>
   </si>
@@ -1018,6 +1161,12 @@
   </si>
   <si>
     <t>PARAM0</t>
+  </si>
+  <si>
+    <t>seed_strategy</t>
+  </si>
+  <si>
+    <t>joint</t>
   </si>
 </sst>
 </file>
@@ -2670,7 +2819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -2724,6 +2873,14 @@
       </c>
       <c r="B6">
         <v>999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>